<commit_message>
data: freeze prover development bank Gate A
</commit_message>
<xml_diff>
--- a/datasets/m2_2b_formal/prover_generator_hardening_v1_2/paired_justification_review12_bilingual.xlsx
+++ b/datasets/m2_2b_formal/prover_generator_hardening_v1_2/paired_justification_review12_bilingual.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="自然化审核v1.2" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="审核说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自然化审核v1.2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1325,7 +1325,7 @@
           <t>A closed access registry uses local status codes. Treat every listed rule as exact and use only the records below. An unlisted statement is not automatically negated.
 Record 1. Account D has status Lilac 5.
 Record 2. Account D has status Cobalt 2.
-Record 3. If an item has status Cobalt 2, then an item has status Jade 3.
+Record 3. If an item has status Cobalt 2, then that same item has status Jade 3.
 Record 4. If Account D has status Amber 1, then it is not the case that Account D has status Ivory 4.
 Record 5. If Account D has status Lilac 5, then Account D has status Copper 6.
 Record 6. If Account D has status Copper 6, then Account D has status Amber 1.
@@ -1337,7 +1337,7 @@
           <t>下面是一份封闭的访问登记簿，其中使用本地状态代码。请严格按照所列规则，且只使用下方记录；未列出的陈述不能自动视为否定。
 记录1：账户丁具有丁香5状态。
 记录2：账户丁具有钴蓝2状态。
-记录3：如果某个对象具有钴蓝2状态，那么某个对象具有碧玉3状态。
+记录3：如果某个对象具有钴蓝2状态，那么该同一对象具有碧玉3状态。
 记录4：如果账户丁具有琥珀1状态，那么并非账户丁具有象牙4状态。
 记录5：如果账户丁具有丁香5状态，那么账户丁具有赤铜6状态。
 记录6：如果账户丁具有赤铜6状态，那么账户丁具有琥珀1状态。
@@ -1396,7 +1396,7 @@
 Record 8. Device C has status Saffron 15.
 Record 9. Device A has status Navy 22.
 Record 10. Device A has status Amber 1.
-Record 11. If an item has status Amber 1, then an item has status Cobalt 2.
+Record 11. If an item has status Amber 1, then that same item has status Cobalt 2.
 Record 12. If it is not the case that Device A has status Navy 22, then Device A has status Jade 3.
 Record 13. If Device A has status Jade 3, then Device A has status Ivory 4.
 Record 14. If Device A has status Ivory 4, then Device A has status Lilac 5.
@@ -1425,7 +1425,7 @@
 记录8：设备丙具有藏红15状态。
 记录9：设备甲具有海军蓝22状态。
 记录10：设备甲具有琥珀1状态。
-记录11：如果某个对象具有琥珀1状态，那么某个对象具有钴蓝2状态。
+记录11：如果某个对象具有琥珀1状态，那么该同一对象具有钴蓝2状态。
 记录12：如果并非设备甲具有海军蓝22状态，那么设备甲具有碧玉3状态。
 记录13：如果设备甲具有碧玉3状态，那么设备甲具有象牙4状态。
 记录14：如果设备甲具有象牙4状态，那么设备甲具有丁香5状态。

</xml_diff>